<commit_message>
Refresh docs, schematics, BOM, and datasheet RAG corpus
</commit_message>
<xml_diff>
--- a/driver_datasheets_and_calculations/BOM.xlsx
+++ b/driver_datasheets_and_calculations/BOM.xlsx
@@ -674,7 +674,7 @@
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -696,7 +696,7 @@
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
@@ -815,7 +815,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M91"/>
+  <dimension ref="A1:M86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2566,7 +2566,7 @@
       </c>
       <c r="M34" s="14" t="inlineStr">
         <is>
-          <t>Gripper valve coil driver; MCP cannot sink coil current.</t>
+          <t>Gripper valve coil driver; GPIO4 cannot sink coil current — use CR1.</t>
         </is>
       </c>
     </row>
@@ -2688,7 +2688,7 @@
       </c>
       <c r="M36" s="14" t="inlineStr">
         <is>
-          <t>Phoenix Contact has NO 5-&gt;3.3 V DIN converter (DC/DC line input &gt;=12 V). Recommended: power WT32-ETH01 from 5 V rail and use its on-board 3.3 V LDO for the MCP23S17; no separate panel 3.3 V supply. If a dedicated 3.3 V rail is required, use a board-mount POL (e.g., Traco TSR-1 / Recom), not Phoenix.</t>
+          <t>Recommended: power WT32-ETH01 from 5 V rail and use its on-board 3.3 V LDO; no separate panel 3.3 V supply. If a dedicated 3.3 V rail is required, use a board-mount POL (e.g., Traco TSR-1 / Recom), not Phoenix.</t>
         </is>
       </c>
     </row>
@@ -4704,7 +4704,7 @@
       <c r="G71" s="12" t="n"/>
       <c r="H71" s="12" t="inlineStr">
         <is>
-          <t>Section — WT32 motion controller (not in drive cabinet)</t>
+          <t>Section — WT32 motion controller (EIP; not in drive cabinet)</t>
         </is>
       </c>
       <c r="I71" s="12" t="n"/>
@@ -4770,7 +4770,7 @@
       </c>
       <c r="M72" s="14" t="inlineStr">
         <is>
-          <t>Gantry firmware; MQTT pick scheduling.</t>
+          <t>Gantry firmware; MQTT pick scheduling over LAN8720.</t>
         </is>
       </c>
     </row>
@@ -4796,22 +4796,22 @@
       </c>
       <c r="F73" s="14" t="inlineStr">
         <is>
-          <t>Microchip</t>
+          <t>WIZnet</t>
         </is>
       </c>
       <c r="G73" s="14" t="inlineStr">
         <is>
-          <t>MCP23S17</t>
+          <t>WIZ850io (W5500)</t>
         </is>
       </c>
       <c r="H73" s="14" t="inlineStr">
         <is>
-          <t>16-bit SPI GPIO expander</t>
+          <t>SPI Ethernet module for EtherNet/IP daisy-chain</t>
         </is>
       </c>
       <c r="I73" s="14" t="inlineStr">
         <is>
-          <t>U1</t>
+          <t>ETH1</t>
         </is>
       </c>
       <c r="J73" s="14" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="M73" s="14" t="inlineStr">
         <is>
-          <t>DIR, ENABLE, ALM, limits, gripper command.</t>
+          <t>EIP originator; SPI pins MOSI12/MISO35/SCLK5/CS15/RST14. See docs/HV_LV_SCHEMATICS.md sheet 06.</t>
         </is>
       </c>
     </row>
@@ -4840,7 +4840,7 @@
       <c r="B74" s="12" t="n"/>
       <c r="C74" s="13" t="inlineStr">
         <is>
-          <t>9.1 Motion I/O interface</t>
+          <t>9.1 Field I/O (EIP)</t>
         </is>
       </c>
       <c r="D74" s="12" t="n"/>
@@ -4849,7 +4849,7 @@
       <c r="G74" s="12" t="n"/>
       <c r="H74" s="12" t="inlineStr">
         <is>
-          <t>Section — opto-isolated WT32/MCP → 24 V drives (see docs/MOTION_IO_INTERFACE.md)</t>
+          <t>Section — drive-side limits + gripper; see docs/EXPECTED_ELECTROMECHANICAL_ASSEMBLY.md</t>
         </is>
       </c>
       <c r="I74" s="12" t="n"/>
@@ -4867,11 +4867,11 @@
       </c>
       <c r="C75" s="14" t="inlineStr">
         <is>
-          <t>Interface</t>
+          <t>Network</t>
         </is>
       </c>
       <c r="D75" s="14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E75" s="14" t="inlineStr">
         <is>
@@ -4880,42 +4880,42 @@
       </c>
       <c r="F75" s="14" t="inlineStr">
         <is>
-          <t>Broadcom / Avago</t>
+          <t>Generic</t>
         </is>
       </c>
       <c r="G75" s="14" t="inlineStr">
         <is>
-          <t>HCPL-2530</t>
+          <t>Cat5e patch cable</t>
         </is>
       </c>
       <c r="H75" s="14" t="inlineStr">
         <is>
-          <t>Dual high-speed optocoupler, transistor output</t>
+          <t>EtherNet/IP daisy-chain jumpers</t>
         </is>
       </c>
       <c r="I75" s="14" t="inlineStr">
         <is>
-          <t>U-IF1..3</t>
+          <t>W-EIP</t>
         </is>
       </c>
       <c r="J75" s="14" t="inlineStr">
         <is>
-          <t>Controller box</t>
-        </is>
-      </c>
-      <c r="K75" s="15" t="inlineStr">
-        <is>
-          <t>Panel design</t>
+          <t>Panel / Machine</t>
+        </is>
+      </c>
+      <c r="K75" s="18" t="inlineStr">
+        <is>
+          <t>Field install</t>
         </is>
       </c>
       <c r="L75" s="14" t="inlineStr">
         <is>
-          <t>Digi-Key / Mouser</t>
+          <t>—</t>
         </is>
       </c>
       <c r="M75" s="14" t="inlineStr">
         <is>
-          <t>One per axis: pulse + direction to K5100 PTI or HCS01 X31.</t>
+          <t>W5500 -&gt; X PORT1; X PORT2 -&gt; Z PORT1; Z PORT2 -&gt; PC uplink (exclusive).</t>
         </is>
       </c>
     </row>
@@ -4928,133 +4928,95 @@
       </c>
       <c r="C76" s="14" t="inlineStr">
         <is>
-          <t>Interface</t>
+          <t>Signal cable</t>
         </is>
       </c>
       <c r="D76" s="14" t="n">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="E76" s="14" t="inlineStr">
         <is>
-          <t>EA</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="F76" s="14" t="inlineStr">
         <is>
-          <t>Vishay / Siliconix</t>
+          <t>Belden</t>
         </is>
       </c>
       <c r="G76" s="14" t="inlineStr">
         <is>
-          <t>VO14642AT</t>
+          <t>8723</t>
         </is>
       </c>
       <c r="H76" s="14" t="inlineStr">
         <is>
-          <t>Phototransistor optocoupler, single channel</t>
+          <t>2-pair 22 AWG individually shielded, 300V</t>
         </is>
       </c>
       <c r="I76" s="14" t="inlineStr">
         <is>
-          <t>U-IF4..8</t>
+          <t>W-LIM</t>
         </is>
       </c>
       <c r="J76" s="14" t="inlineStr">
         <is>
-          <t>Controller box</t>
-        </is>
-      </c>
-      <c r="K76" s="15" t="inlineStr">
-        <is>
-          <t>Panel design</t>
+          <t>Machine</t>
+        </is>
+      </c>
+      <c r="K76" s="18" t="inlineStr">
+        <is>
+          <t>Field install</t>
         </is>
       </c>
       <c r="L76" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Belden 8723</t>
         </is>
       </c>
       <c r="M76" s="14" t="inlineStr">
         <is>
-          <t>X SON+ARST, Z SON+ARST, Theta enable. No dual-channel SKU.</t>
+          <t>NC limit switches to TBIO INPUT1-4 / HCS01 X31.5-6 (not ESP32).</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="14" t="n">
-        <v>64</v>
-      </c>
-      <c r="B77" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C77" s="14" t="inlineStr">
-        <is>
-          <t>Interface</t>
-        </is>
-      </c>
-      <c r="D77" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="E77" s="14" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="F77" s="14" t="inlineStr">
-        <is>
-          <t>Broadcom / Avago</t>
-        </is>
-      </c>
-      <c r="G77" s="14" t="inlineStr">
-        <is>
-          <t>HCPL-3700</t>
-        </is>
-      </c>
-      <c r="H77" s="14" t="inlineStr">
-        <is>
-          <t>Line-voltage threshold detector opto</t>
-        </is>
-      </c>
-      <c r="I77" s="14" t="inlineStr">
-        <is>
-          <t>U-IF9..10</t>
-        </is>
-      </c>
-      <c r="J77" s="14" t="inlineStr">
-        <is>
-          <t>Controller box</t>
-        </is>
-      </c>
-      <c r="K77" s="15" t="inlineStr">
-        <is>
-          <t>Panel design</t>
-        </is>
-      </c>
-      <c r="L77" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M77" s="14" t="inlineStr">
-        <is>
-          <t>K5100 ALM → MCP for X and Z.</t>
-        </is>
-      </c>
+      <c r="A77" s="12" t="n"/>
+      <c r="B77" s="12" t="n"/>
+      <c r="C77" s="13" t="inlineStr">
+        <is>
+          <t>10.0 Field wiring</t>
+        </is>
+      </c>
+      <c r="D77" s="12" t="n"/>
+      <c r="E77" s="12" t="n"/>
+      <c r="F77" s="12" t="n"/>
+      <c r="G77" s="12" t="n"/>
+      <c r="H77" s="12" t="inlineStr">
+        <is>
+          <t>Section — cables &amp; harnesses (not panel-mounted)</t>
+        </is>
+      </c>
+      <c r="I77" s="12" t="n"/>
+      <c r="J77" s="12" t="n"/>
+      <c r="K77" s="12" t="n"/>
+      <c r="L77" s="12" t="n"/>
+      <c r="M77" s="12" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="14" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B78" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C78" s="14" t="inlineStr">
         <is>
-          <t>Interface</t>
+          <t>Field cable</t>
         </is>
       </c>
       <c r="D78" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E78" s="14" t="inlineStr">
         <is>
@@ -5063,55 +5025,55 @@
       </c>
       <c r="F78" s="14" t="inlineStr">
         <is>
-          <t>TI</t>
+          <t>Allen-Bradley</t>
         </is>
       </c>
       <c r="G78" s="14" t="inlineStr">
         <is>
-          <t>SN74AHCT244</t>
+          <t>2090-CPWM7DF-16AF03</t>
         </is>
       </c>
       <c r="H78" s="14" t="inlineStr">
         <is>
-          <t>Octal buffer, 5 V, drives opto LEDs from 3.3 V logic</t>
+          <t>Motor power cable, 16 AWG, 3 m, continuous-flex</t>
         </is>
       </c>
       <c r="I78" s="14" t="inlineStr">
         <is>
-          <t>U-IF11..12</t>
+          <t>W1</t>
         </is>
       </c>
       <c r="J78" s="14" t="inlineStr">
         <is>
-          <t>Controller box</t>
-        </is>
-      </c>
-      <c r="K78" s="15" t="inlineStr">
-        <is>
-          <t>Panel design</t>
+          <t>Machine</t>
+        </is>
+      </c>
+      <c r="K78" s="16" t="inlineStr">
+        <is>
+          <t>On order</t>
         </is>
       </c>
       <c r="L78" s="14" t="inlineStr">
         <is>
-          <t>TI</t>
+          <t>McMc P0078269 L6</t>
         </is>
       </c>
       <c r="M78" s="14" t="inlineStr">
         <is>
-          <t>11 gates used; 3.3 V tolerant inputs.</t>
+          <t>DRV1 &lt;-&gt; MPL-A320P.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="14" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B79" s="14" t="n">
         <v>1</v>
       </c>
       <c r="C79" s="14" t="inlineStr">
         <is>
-          <t>Interface</t>
+          <t>Field cable</t>
         </is>
       </c>
       <c r="D79" s="14" t="n">
@@ -5124,128 +5086,166 @@
       </c>
       <c r="F79" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Allen-Bradley</t>
         </is>
       </c>
       <c r="G79" s="14" t="inlineStr">
         <is>
-          <t>5 VDC regulator module</t>
+          <t>2090-CFBM7DF-CEAF03</t>
         </is>
       </c>
       <c r="H79" s="14" t="inlineStr">
         <is>
-          <t>LM2596 or 7805 class, 24 V in / 5 V out, ~300 mA</t>
+          <t>Motor feedback cable, 3 m</t>
         </is>
       </c>
       <c r="I79" s="14" t="inlineStr">
         <is>
-          <t>PS-IF1</t>
+          <t>W2</t>
         </is>
       </c>
       <c r="J79" s="14" t="inlineStr">
         <is>
-          <t>Controller box</t>
-        </is>
-      </c>
-      <c r="K79" s="15" t="inlineStr">
-        <is>
-          <t>Panel design</t>
+          <t>Machine</t>
+        </is>
+      </c>
+      <c r="K79" s="16" t="inlineStr">
+        <is>
+          <t>On order</t>
         </is>
       </c>
       <c r="L79" s="14" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>McMc P0078269 L7</t>
         </is>
       </c>
       <c r="M79" s="14" t="inlineStr">
         <is>
-          <t>Powers 74AHCT244 and opto LED side. LOGIC_GND.</t>
+          <t>DRV1 &lt;-&gt; MPL encoder.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="14" t="n">
+        <v>66</v>
+      </c>
+      <c r="B80" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C80" s="14" t="inlineStr">
+        <is>
+          <t>Field cable</t>
+        </is>
+      </c>
+      <c r="D80" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E80" s="14" t="inlineStr">
+        <is>
+          <t>EA</t>
+        </is>
+      </c>
+      <c r="F80" s="14" t="inlineStr">
+        <is>
+          <t>Allen-Bradley</t>
+        </is>
+      </c>
+      <c r="G80" s="14" t="inlineStr">
+        <is>
+          <t>2090-CPWM7DF-16AF03</t>
+        </is>
+      </c>
+      <c r="H80" s="14" t="inlineStr">
+        <is>
+          <t>Motor power cable, 16 AWG, 3 m, continuous-flex</t>
+        </is>
+      </c>
+      <c r="I80" s="14" t="inlineStr">
+        <is>
+          <t>W3</t>
+        </is>
+      </c>
+      <c r="J80" s="14" t="inlineStr">
+        <is>
+          <t>Machine</t>
+        </is>
+      </c>
+      <c r="K80" s="16" t="inlineStr">
+        <is>
+          <t>On order</t>
+        </is>
+      </c>
+      <c r="L80" s="14" t="inlineStr">
+        <is>
+          <t>McMc P0078269 L14</t>
+        </is>
+      </c>
+      <c r="M80" s="14" t="inlineStr">
+        <is>
+          <t>DRV2 &lt;-&gt; MPL-A310F.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="14" t="n">
         <v>67</v>
       </c>
-      <c r="B80" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C80" s="14" t="inlineStr">
-        <is>
-          <t>Interface</t>
-        </is>
-      </c>
-      <c r="D80" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E80" s="14" t="inlineStr">
+      <c r="B81" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C81" s="14" t="inlineStr">
+        <is>
+          <t>Field cable</t>
+        </is>
+      </c>
+      <c r="D81" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E81" s="14" t="inlineStr">
         <is>
           <t>EA</t>
         </is>
       </c>
-      <c r="F80" s="14" t="inlineStr">
-        <is>
-          <t>Wago / Phoenix</t>
-        </is>
-      </c>
-      <c r="G80" s="14" t="inlineStr">
-        <is>
-          <t>Terminal block set</t>
-        </is>
-      </c>
-      <c r="H80" s="14" t="inlineStr">
-        <is>
-          <t>Logic-side + field-side harness landing</t>
-        </is>
-      </c>
-      <c r="I80" s="14" t="inlineStr">
-        <is>
-          <t>TB-IF</t>
-        </is>
-      </c>
-      <c r="J80" s="14" t="inlineStr">
-        <is>
-          <t>Controller box</t>
-        </is>
-      </c>
-      <c r="K80" s="15" t="inlineStr">
-        <is>
-          <t>Panel design</t>
-        </is>
-      </c>
-      <c r="L80" s="14" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M80" s="14" t="inlineStr">
-        <is>
-          <t>Star FIELD_0V here; shields at drive end only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" s="12" t="n"/>
-      <c r="B81" s="12" t="n"/>
-      <c r="C81" s="13" t="inlineStr">
-        <is>
-          <t>10.0 Field wiring</t>
-        </is>
-      </c>
-      <c r="D81" s="12" t="n"/>
-      <c r="E81" s="12" t="n"/>
-      <c r="F81" s="12" t="n"/>
-      <c r="G81" s="12" t="n"/>
-      <c r="H81" s="12" t="inlineStr">
-        <is>
-          <t>Section — cables &amp; harnesses (not panel-mounted)</t>
-        </is>
-      </c>
-      <c r="I81" s="12" t="n"/>
-      <c r="J81" s="12" t="n"/>
-      <c r="K81" s="12" t="n"/>
-      <c r="L81" s="12" t="n"/>
-      <c r="M81" s="12" t="n"/>
+      <c r="F81" s="14" t="inlineStr">
+        <is>
+          <t>Allen-Bradley</t>
+        </is>
+      </c>
+      <c r="G81" s="14" t="inlineStr">
+        <is>
+          <t>2090-CFBM7DF-CEAF03</t>
+        </is>
+      </c>
+      <c r="H81" s="14" t="inlineStr">
+        <is>
+          <t>Motor feedback cable, 3 m</t>
+        </is>
+      </c>
+      <c r="I81" s="14" t="inlineStr">
+        <is>
+          <t>W4</t>
+        </is>
+      </c>
+      <c r="J81" s="14" t="inlineStr">
+        <is>
+          <t>Machine</t>
+        </is>
+      </c>
+      <c r="K81" s="16" t="inlineStr">
+        <is>
+          <t>On order</t>
+        </is>
+      </c>
+      <c r="L81" s="14" t="inlineStr">
+        <is>
+          <t>McMc P0078269 L15</t>
+        </is>
+      </c>
+      <c r="M81" s="14" t="inlineStr">
+        <is>
+          <t>DRV2 &lt;-&gt; MPL encoder.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="14" t="n">
@@ -5269,22 +5269,22 @@
       </c>
       <c r="F82" s="14" t="inlineStr">
         <is>
-          <t>Allen-Bradley</t>
+          <t>SCHUNK</t>
         </is>
       </c>
       <c r="G82" s="14" t="inlineStr">
         <is>
-          <t>2090-CPWM7DF-16AF03</t>
+          <t>KA GLT1706-LK-00500-1</t>
         </is>
       </c>
       <c r="H82" s="14" t="inlineStr">
         <is>
-          <t>Motor power cable, 16 AWG, 3 m, continuous-flex</t>
+          <t>ERD motor power cable, 5 m</t>
         </is>
       </c>
       <c r="I82" s="14" t="inlineStr">
         <is>
-          <t>W1</t>
+          <t>W5</t>
         </is>
       </c>
       <c r="J82" s="14" t="inlineStr">
@@ -5299,12 +5299,12 @@
       </c>
       <c r="L82" s="14" t="inlineStr">
         <is>
-          <t>McMc P0078269 L6</t>
+          <t>Youngblood 349-104</t>
         </is>
       </c>
       <c r="M82" s="14" t="inlineStr">
         <is>
-          <t>DRV1 ↔ MPL-A320P.</t>
+          <t>DRV3 &lt;-&gt; ERD — factory cable.</t>
         </is>
       </c>
     </row>
@@ -5330,22 +5330,22 @@
       </c>
       <c r="F83" s="14" t="inlineStr">
         <is>
-          <t>Allen-Bradley</t>
+          <t>SCHUNK</t>
         </is>
       </c>
       <c r="G83" s="14" t="inlineStr">
         <is>
-          <t>2090-CFBM7DF-CEAF03</t>
+          <t>KA WWN1208-GK-00500-K02</t>
         </is>
       </c>
       <c r="H83" s="14" t="inlineStr">
         <is>
-          <t>Motor feedback cable, 3 m</t>
+          <t>ERD HIPERFACE encoder cable, 5 m</t>
         </is>
       </c>
       <c r="I83" s="14" t="inlineStr">
         <is>
-          <t>W2</t>
+          <t>W6</t>
         </is>
       </c>
       <c r="J83" s="14" t="inlineStr">
@@ -5360,12 +5360,12 @@
       </c>
       <c r="L83" s="14" t="inlineStr">
         <is>
-          <t>McMc P0078269 L7</t>
+          <t>Youngblood 349-544</t>
         </is>
       </c>
       <c r="M83" s="14" t="inlineStr">
         <is>
-          <t>DRV1 ↔ MPL encoder.</t>
+          <t>DRV3 &lt;-&gt; ERD feedback.</t>
         </is>
       </c>
     </row>
@@ -5378,55 +5378,55 @@
       </c>
       <c r="C84" s="14" t="inlineStr">
         <is>
-          <t>Field cable</t>
+          <t>Panel wire</t>
         </is>
       </c>
       <c r="D84" s="14" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="E84" s="14" t="inlineStr">
         <is>
-          <t>EA</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="F84" s="14" t="inlineStr">
         <is>
-          <t>Allen-Bradley</t>
+          <t>Lapp / LappUSA</t>
         </is>
       </c>
       <c r="G84" s="14" t="inlineStr">
         <is>
-          <t>2090-CPWM7DF-16AF03</t>
+          <t>OLFLEX WIRE MS 2.1, 10 mm2 (UL MTW/1015 600V)</t>
         </is>
       </c>
       <c r="H84" s="14" t="inlineStr">
         <is>
-          <t>Motor power cable, 16 AWG, 3 m, continuous-flex</t>
+          <t>8 AWG MTW single conductor (BK/BR/OR + GN-PE)</t>
         </is>
       </c>
       <c r="I84" s="14" t="inlineStr">
         <is>
-          <t>W3</t>
+          <t>W-X</t>
         </is>
       </c>
       <c r="J84" s="14" t="inlineStr">
         <is>
-          <t>Machine</t>
-        </is>
-      </c>
-      <c r="K84" s="16" t="inlineStr">
-        <is>
-          <t>On order</t>
+          <t>Panel</t>
+        </is>
+      </c>
+      <c r="K84" s="18" t="inlineStr">
+        <is>
+          <t>Field install</t>
         </is>
       </c>
       <c r="L84" s="14" t="inlineStr">
         <is>
-          <t>McMc P0078269 L14</t>
+          <t>Lapp 4160-series</t>
         </is>
       </c>
       <c r="M84" s="14" t="inlineStr">
         <is>
-          <t>DRV2 ↔ MPL-A310F.</t>
+          <t>X 40 A branch + CB0 feeder. NEC 430.122: conductor &gt;= 125% of drive INPUT FLC = 1.25 x 11.6 = 14.5 A (8 AWG is conservative; NEC min would be 14 AWG). 13.4 A is the drive OUTPUT, not the branch load. Not in inventory.</t>
         </is>
       </c>
     </row>
@@ -5439,55 +5439,55 @@
       </c>
       <c r="C85" s="14" t="inlineStr">
         <is>
-          <t>Field cable</t>
+          <t>Panel wire</t>
         </is>
       </c>
       <c r="D85" s="14" t="n">
-        <v>1</v>
+        <v>120</v>
       </c>
       <c r="E85" s="14" t="inlineStr">
         <is>
-          <t>EA</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="F85" s="14" t="inlineStr">
         <is>
-          <t>Allen-Bradley</t>
+          <t>Lapp / LappUSA</t>
         </is>
       </c>
       <c r="G85" s="14" t="inlineStr">
         <is>
-          <t>2090-CFBM7DF-CEAF03</t>
+          <t>OLFLEX WIRE MS 2.1, 1.5 mm2 (UL MTW/1015 600V)</t>
         </is>
       </c>
       <c r="H85" s="14" t="inlineStr">
         <is>
-          <t>Motor feedback cable, 3 m</t>
+          <t>16 AWG MTW single conductor (BK/BR/OR + GN-PE)</t>
         </is>
       </c>
       <c r="I85" s="14" t="inlineStr">
         <is>
-          <t>W4</t>
+          <t>W-AC16</t>
         </is>
       </c>
       <c r="J85" s="14" t="inlineStr">
         <is>
-          <t>Machine</t>
-        </is>
-      </c>
-      <c r="K85" s="16" t="inlineStr">
-        <is>
-          <t>On order</t>
+          <t>Panel</t>
+        </is>
+      </c>
+      <c r="K85" s="19" t="inlineStr">
+        <is>
+          <t>On hand</t>
         </is>
       </c>
       <c r="L85" s="14" t="inlineStr">
         <is>
-          <t>McMc P0078269 L15</t>
+          <t>Lapp 4160-series</t>
         </is>
       </c>
       <c r="M85" s="14" t="inlineStr">
         <is>
-          <t>DRV2 ↔ MPL encoder.</t>
+          <t>Z + Theta + PSU AC branches. 80%: 16 AWG cap 10 A OCPD -&gt; 8 A cont &gt;= 2.6/2.0/1.2 A loads.</t>
         </is>
       </c>
     </row>
@@ -5500,360 +5500,55 @@
       </c>
       <c r="C86" s="14" t="inlineStr">
         <is>
-          <t>Field cable</t>
+          <t>Panel wire</t>
         </is>
       </c>
       <c r="D86" s="14" t="n">
-        <v>1</v>
+        <v>80</v>
       </c>
       <c r="E86" s="14" t="inlineStr">
         <is>
-          <t>EA</t>
+          <t>FT</t>
         </is>
       </c>
       <c r="F86" s="14" t="inlineStr">
         <is>
-          <t>SCHUNK</t>
+          <t>Lapp / LappUSA</t>
         </is>
       </c>
       <c r="G86" s="14" t="inlineStr">
         <is>
-          <t>KA GLT1706-LK-00500-1</t>
+          <t>OLFLEX WIRE MS 2.1, 1.0 mm2 (UL MTW/1015 600V)</t>
         </is>
       </c>
       <c r="H86" s="14" t="inlineStr">
         <is>
-          <t>ERD motor power cable, 5 m</t>
+          <t>18 AWG MTW single conductor (RD +24V, BU 0V, YE e-stop, WT)</t>
         </is>
       </c>
       <c r="I86" s="14" t="inlineStr">
         <is>
-          <t>W5</t>
+          <t>W-DC18</t>
         </is>
       </c>
       <c r="J86" s="14" t="inlineStr">
         <is>
-          <t>Machine</t>
-        </is>
-      </c>
-      <c r="K86" s="16" t="inlineStr">
-        <is>
-          <t>On order</t>
+          <t>Panel</t>
+        </is>
+      </c>
+      <c r="K86" s="19" t="inlineStr">
+        <is>
+          <t>On hand</t>
         </is>
       </c>
       <c r="L86" s="14" t="inlineStr">
         <is>
-          <t>Youngblood 349-104</t>
+          <t>Lapp 4160-series</t>
         </is>
       </c>
       <c r="M86" s="14" t="inlineStr">
         <is>
-          <t>DRV3 ↔ ERD — factory cable.</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="14" t="n">
-        <v>73</v>
-      </c>
-      <c r="B87" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C87" s="14" t="inlineStr">
-        <is>
-          <t>Field cable</t>
-        </is>
-      </c>
-      <c r="D87" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E87" s="14" t="inlineStr">
-        <is>
-          <t>EA</t>
-        </is>
-      </c>
-      <c r="F87" s="14" t="inlineStr">
-        <is>
-          <t>SCHUNK</t>
-        </is>
-      </c>
-      <c r="G87" s="14" t="inlineStr">
-        <is>
-          <t>KA WWN1208-GK-00500-K02</t>
-        </is>
-      </c>
-      <c r="H87" s="14" t="inlineStr">
-        <is>
-          <t>ERD HIPERFACE encoder cable, 5 m</t>
-        </is>
-      </c>
-      <c r="I87" s="14" t="inlineStr">
-        <is>
-          <t>W6</t>
-        </is>
-      </c>
-      <c r="J87" s="14" t="inlineStr">
-        <is>
-          <t>Machine</t>
-        </is>
-      </c>
-      <c r="K87" s="16" t="inlineStr">
-        <is>
-          <t>On order</t>
-        </is>
-      </c>
-      <c r="L87" s="14" t="inlineStr">
-        <is>
-          <t>Youngblood 349-544</t>
-        </is>
-      </c>
-      <c r="M87" s="14" t="inlineStr">
-        <is>
-          <t>DRV3 ↔ ERD feedback.</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="14" t="n">
-        <v>74</v>
-      </c>
-      <c r="B88" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C88" s="14" t="inlineStr">
-        <is>
-          <t>Panel wire</t>
-        </is>
-      </c>
-      <c r="D88" s="14" t="n">
-        <v>60</v>
-      </c>
-      <c r="E88" s="14" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="F88" s="14" t="inlineStr">
-        <is>
-          <t>Lapp / LappUSA</t>
-        </is>
-      </c>
-      <c r="G88" s="14" t="inlineStr">
-        <is>
-          <t>OLFLEX WIRE MS 2.1, 10 mm2 (UL MTW/1015 600V)</t>
-        </is>
-      </c>
-      <c r="H88" s="14" t="inlineStr">
-        <is>
-          <t>8 AWG MTW single conductor (BK/BR/OR + GN-PE)</t>
-        </is>
-      </c>
-      <c r="I88" s="14" t="inlineStr">
-        <is>
-          <t>W-X</t>
-        </is>
-      </c>
-      <c r="J88" s="14" t="inlineStr">
-        <is>
-          <t>Panel</t>
-        </is>
-      </c>
-      <c r="K88" s="18" t="inlineStr">
-        <is>
-          <t>Field install</t>
-        </is>
-      </c>
-      <c r="L88" s="14" t="inlineStr">
-        <is>
-          <t>Lapp 4160-series</t>
-        </is>
-      </c>
-      <c r="M88" s="14" t="inlineStr">
-        <is>
-          <t>X 40 A branch + CB0 feeder. NEC 430.122: conductor &gt;= 125% of drive INPUT FLC = 1.25 x 11.6 = 14.5 A (8 AWG is conservative; NEC min would be 14 AWG). 13.4 A is the drive OUTPUT, not the branch load. Not in inventory.</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="14" t="n">
-        <v>75</v>
-      </c>
-      <c r="B89" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C89" s="14" t="inlineStr">
-        <is>
-          <t>Panel wire</t>
-        </is>
-      </c>
-      <c r="D89" s="14" t="n">
-        <v>120</v>
-      </c>
-      <c r="E89" s="14" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="F89" s="14" t="inlineStr">
-        <is>
-          <t>Lapp / LappUSA</t>
-        </is>
-      </c>
-      <c r="G89" s="14" t="inlineStr">
-        <is>
-          <t>OLFLEX WIRE MS 2.1, 1.5 mm2 (UL MTW/1015 600V)</t>
-        </is>
-      </c>
-      <c r="H89" s="14" t="inlineStr">
-        <is>
-          <t>16 AWG MTW single conductor (BK/BR/OR + GN-PE)</t>
-        </is>
-      </c>
-      <c r="I89" s="14" t="inlineStr">
-        <is>
-          <t>W-AC16</t>
-        </is>
-      </c>
-      <c r="J89" s="14" t="inlineStr">
-        <is>
-          <t>Panel</t>
-        </is>
-      </c>
-      <c r="K89" s="19" t="inlineStr">
-        <is>
-          <t>On hand</t>
-        </is>
-      </c>
-      <c r="L89" s="14" t="inlineStr">
-        <is>
-          <t>Lapp 4160-series</t>
-        </is>
-      </c>
-      <c r="M89" s="14" t="inlineStr">
-        <is>
-          <t>Z + Theta + PSU AC branches. 80%: 16 AWG cap 10 A OCPD -&gt; 8 A cont &gt;= 2.6/2.0/1.2 A loads.</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="14" t="n">
-        <v>76</v>
-      </c>
-      <c r="B90" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C90" s="14" t="inlineStr">
-        <is>
-          <t>Panel wire</t>
-        </is>
-      </c>
-      <c r="D90" s="14" t="n">
-        <v>80</v>
-      </c>
-      <c r="E90" s="14" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="F90" s="14" t="inlineStr">
-        <is>
-          <t>Lapp / LappUSA</t>
-        </is>
-      </c>
-      <c r="G90" s="14" t="inlineStr">
-        <is>
-          <t>OLFLEX WIRE MS 2.1, 1.0 mm2 (UL MTW/1015 600V)</t>
-        </is>
-      </c>
-      <c r="H90" s="14" t="inlineStr">
-        <is>
-          <t>18 AWG MTW single conductor (RD +24V, BU 0V, YE e-stop, WT)</t>
-        </is>
-      </c>
-      <c r="I90" s="14" t="inlineStr">
-        <is>
-          <t>W-DC18</t>
-        </is>
-      </c>
-      <c r="J90" s="14" t="inlineStr">
-        <is>
-          <t>Panel</t>
-        </is>
-      </c>
-      <c r="K90" s="19" t="inlineStr">
-        <is>
-          <t>On hand</t>
-        </is>
-      </c>
-      <c r="L90" s="14" t="inlineStr">
-        <is>
-          <t>Lapp 4160-series</t>
-        </is>
-      </c>
-      <c r="M90" s="14" t="inlineStr">
-        <is>
           <t>24 VDC bus, E-stop chain, gripper valve coil. 80%: 18 AWG 7 A OCPD -&gt; 5.6 A cont &gt;= ~3 A.</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="14" t="n">
-        <v>77</v>
-      </c>
-      <c r="B91" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C91" s="14" t="inlineStr">
-        <is>
-          <t>Signal cable</t>
-        </is>
-      </c>
-      <c r="D91" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="E91" s="14" t="inlineStr">
-        <is>
-          <t>FT</t>
-        </is>
-      </c>
-      <c r="F91" s="14" t="inlineStr">
-        <is>
-          <t>Belden</t>
-        </is>
-      </c>
-      <c r="G91" s="14" t="inlineStr">
-        <is>
-          <t>8723</t>
-        </is>
-      </c>
-      <c r="H91" s="14" t="inlineStr">
-        <is>
-          <t>2-pair 22 AWG individually shielded, 300V</t>
-        </is>
-      </c>
-      <c r="I91" s="14" t="inlineStr">
-        <is>
-          <t>W-SIG</t>
-        </is>
-      </c>
-      <c r="J91" s="14" t="inlineStr">
-        <is>
-          <t>Controller box</t>
-        </is>
-      </c>
-      <c r="K91" s="18" t="inlineStr">
-        <is>
-          <t>Field install</t>
-        </is>
-      </c>
-      <c r="L91" s="14" t="inlineStr">
-        <is>
-          <t>Belden 8723</t>
-        </is>
-      </c>
-      <c r="M91" s="14" t="inlineStr">
-        <is>
-          <t>PTI/DIR/EN/ALM/limits/SPI: WT32/MCP -&gt; TB1/TB2/HCS01. See WIRE_SIZE_SELECTION.xlsx.</t>
         </is>
       </c>
     </row>
@@ -8947,7 +8642,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8961,7 +8656,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Control signal reference (WT32-ETH01 / MCP23S17)</t>
+          <t>Control signal reference (WT32-ETH01 / W5500 EIP)</t>
         </is>
       </c>
     </row>
@@ -9000,113 +8695,113 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>PTI X</t>
+          <t>EIP O→T / T→O</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>WT32 GPIO14</t>
+          <t>W5500</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>TB1 (DRV1)</t>
+          <t>Kinetix X/Z</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>22 AWG STP</t>
+          <t>Cat5e+</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>PIN_X_PULSE</t>
+          <t>104 / 154</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>LEDC pulse train</t>
+          <t>Class 1 RPI 5 ms</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>PTI Z</t>
+          <t>EIP daisy continue</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>WT32 GPIO2</t>
+          <t>X PORT2</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>TB2 (DRV2)</t>
+          <t>Z PORT1</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>22 AWG STP</t>
+          <t>Cat5e+</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>PIN_Z_PULSE</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Boot strap — LOW at reset</t>
+          <t>Then Z PORT2 → PC</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>PTI Theta</t>
+          <t>W5500 SPI</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>WT32 GPIO0</t>
+          <t>WT32</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>DRV3</t>
+          <t>WIZ850io</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>22 AWG STP</t>
+          <t>short harness</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>PIN_THETA_PULSE</t>
+          <t>12/35/5/15/14</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Boot strap — HIGH at reset</t>
+          <t>MOSI/MISO/SCLK/CS/RST</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>DIR / EN / ALM</t>
+          <t>Limits X</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>MCP23S17</t>
+          <t>Beta 100-ZRS</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>TB1 / TB2 / DRV3</t>
+          <t>TBIO INPUT1/2</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -9116,29 +8811,29 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>PIN_*</t>
+          <t>pins 9/10</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Digital I/O</t>
+          <t>NC sinking</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Limits</t>
+          <t>Limits Z</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Beta actuators</t>
+          <t>Beta 80-SRS</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>MCP23S17</t>
+          <t>TBIO INPUT3/4</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -9148,12 +8843,12 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>PIN_*_LIMIT_*</t>
+          <t>pins 34/8</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Homing / abort</t>
+          <t>NC sinking</t>
         </is>
       </c>
     </row>
@@ -9165,12 +8860,12 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>MCP A.7</t>
+          <t>GPIO4</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>CR1 coil</t>
+          <t>CR1 coil → SV1</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -9192,64 +8887,32 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>MCP SPI</t>
+          <t>MQTT Ethernet</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>WT32</t>
+          <t>WT32 LAN8720</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>MCP23S17</t>
+          <t>Plant network</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>2-pair 22 AWG</t>
+          <t>Cat5e/6</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>CS/MOSI/MISO/SCLK</t>
+          <t>—</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>&lt;0.5 m</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>Ethernet</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>WT32</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>Plant network</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>Cat5e/6</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>MQTT</t>
+          <t>Separate from EIP</t>
         </is>
       </c>
     </row>

</xml_diff>